<commit_message>
Add Power BI effort estimate tab and option comparison
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019bpAoRK7hQgLeuTSRxMupp
</commit_message>
<xml_diff>
--- a/docs/SRD_effort_estimate.xlsx
+++ b/docs/SRD_effort_estimate.xlsx
@@ -8,9 +8,10 @@
   </bookViews>
   <sheets>
     <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Effort Estimate" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Assumptions" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Requirement Mapping" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Power BI Estimate" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Effort Estimate" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Assumptions" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Requirement Mapping" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,9 +21,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="#,##0;(#,##0);-"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="164" formatCode="#,##0;(#,##0);-"/>
+    <numFmt numFmtId="165" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -122,17 +123,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -140,28 +141,28 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -179,6 +180,28 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -545,10 +568,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
@@ -564,7 +587,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Metric</t>
+          <t>Option A: Streamlit/Python (incl. data layer)</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -589,15 +612,15 @@
           <t>Base effort (hours)</t>
         </is>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="25">
         <f>'Effort Estimate'!E18</f>
         <v/>
       </c>
-      <c r="C4" s="4">
+      <c r="C4" s="25">
         <f>'Effort Estimate'!F18</f>
         <v/>
       </c>
-      <c r="D4" s="4">
+      <c r="D4" s="25">
         <f>'Effort Estimate'!G18</f>
         <v/>
       </c>
@@ -608,15 +631,15 @@
           <t>Contingency buffer (hours)</t>
         </is>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="25">
         <f>'Effort Estimate'!E19</f>
         <v/>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="25">
         <f>'Effort Estimate'!F19</f>
         <v/>
       </c>
-      <c r="D5" s="4">
+      <c r="D5" s="25">
         <f>'Effort Estimate'!G19</f>
         <v/>
       </c>
@@ -627,15 +650,15 @@
           <t>Total with buffer (hours)</t>
         </is>
       </c>
-      <c r="B6" s="6">
+      <c r="B6" s="26">
         <f>'Effort Estimate'!E20</f>
         <v/>
       </c>
-      <c r="C6" s="6">
+      <c r="C6" s="26">
         <f>'Effort Estimate'!F20</f>
         <v/>
       </c>
-      <c r="D6" s="6">
+      <c r="D6" s="26">
         <f>'Effort Estimate'!G20</f>
         <v/>
       </c>
@@ -646,15 +669,15 @@
           <t>Working days</t>
         </is>
       </c>
-      <c r="B7" s="7">
+      <c r="B7" s="27">
         <f>B6/(Assumptions!$B$4*Assumptions!$B$6)</f>
         <v/>
       </c>
-      <c r="C7" s="7">
+      <c r="C7" s="27">
         <f>C6/(Assumptions!$B$4*Assumptions!$B$6)</f>
         <v/>
       </c>
-      <c r="D7" s="7">
+      <c r="D7" s="27">
         <f>D6/(Assumptions!$B$4*Assumptions!$B$6)</f>
         <v/>
       </c>
@@ -665,15 +688,15 @@
           <t>Calendar weeks</t>
         </is>
       </c>
-      <c r="B8" s="7">
+      <c r="B8" s="27">
         <f>B6/(Assumptions!$B$5*Assumptions!$B$6)</f>
         <v/>
       </c>
-      <c r="C8" s="7">
+      <c r="C8" s="27">
         <f>C6/(Assumptions!$B$5*Assumptions!$B$6)</f>
         <v/>
       </c>
-      <c r="D8" s="7">
+      <c r="D8" s="27">
         <f>D6/(Assumptions!$B$5*Assumptions!$B$6)</f>
         <v/>
       </c>
@@ -684,28 +707,182 @@
           <t>Cost (INR)</t>
         </is>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="25">
         <f>B6*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="25">
         <f>C6*Assumptions!$B$7</f>
         <v/>
       </c>
-      <c r="D9" s="4">
+      <c r="D9" s="25">
         <f>D6*Assumptions!$B$7</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
-        <is>
-          <t>Sheets: Effort Estimate (work packages) | Requirement Mapping (gaps vs. existing app) | Assumptions (buffer, rates, risks).</t>
+      <c r="A11" s="23" t="inlineStr">
+        <is>
+          <t>Option B: Power BI on PostgreSQL DWH (client provides data up to DWH)</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Best case</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Estimated</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Worst case</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Base effort (hours)</t>
+        </is>
+      </c>
+      <c r="B13" s="25">
+        <f>'Power BI Estimate'!E18</f>
+        <v/>
+      </c>
+      <c r="C13" s="25">
+        <f>'Power BI Estimate'!F18</f>
+        <v/>
+      </c>
+      <c r="D13" s="25">
+        <f>'Power BI Estimate'!G18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Contingency buffer (hours)</t>
+        </is>
+      </c>
+      <c r="B14" s="25">
+        <f>'Power BI Estimate'!E19</f>
+        <v/>
+      </c>
+      <c r="C14" s="25">
+        <f>'Power BI Estimate'!F19</f>
+        <v/>
+      </c>
+      <c r="D14" s="25">
+        <f>'Power BI Estimate'!G19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>Total with buffer (hours)</t>
+        </is>
+      </c>
+      <c r="B15" s="26">
+        <f>'Power BI Estimate'!E20</f>
+        <v/>
+      </c>
+      <c r="C15" s="26">
+        <f>'Power BI Estimate'!F20</f>
+        <v/>
+      </c>
+      <c r="D15" s="26">
+        <f>'Power BI Estimate'!G20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Working days</t>
+        </is>
+      </c>
+      <c r="B16" s="27">
+        <f>B15/(Assumptions!$B$4*Assumptions!$B$6)</f>
+        <v/>
+      </c>
+      <c r="C16" s="27">
+        <f>C15/(Assumptions!$B$4*Assumptions!$B$6)</f>
+        <v/>
+      </c>
+      <c r="D16" s="27">
+        <f>D15/(Assumptions!$B$4*Assumptions!$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Calendar weeks</t>
+        </is>
+      </c>
+      <c r="B17" s="27">
+        <f>B15/(Assumptions!$B$5*Assumptions!$B$6)</f>
+        <v/>
+      </c>
+      <c r="C17" s="27">
+        <f>C15/(Assumptions!$B$5*Assumptions!$B$6)</f>
+        <v/>
+      </c>
+      <c r="D17" s="27">
+        <f>D15/(Assumptions!$B$5*Assumptions!$B$6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Cost (INR)</t>
+        </is>
+      </c>
+      <c r="B18" s="25">
+        <f>B15*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="C18" s="25">
+        <f>C15*Assumptions!$B$7</f>
+        <v/>
+      </c>
+      <c r="D18" s="25">
+        <f>D15*Assumptions!$B$7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="23" t="inlineStr">
+        <is>
+          <t>Difference: Option B vs Option A (total hours, estimated)</t>
+        </is>
+      </c>
+      <c r="C20" s="28">
+        <f>C15-C6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Sheets: Effort Estimate (Option A) | Power BI Estimate (Option B) | Requirement Mapping | Assumptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
         <is>
           <t>Cost is 0 until a rate is entered in Assumptions!B7.</t>
         </is>
@@ -717,6 +894,648 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="70" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>SRD Logistics - Power BI Delivery (Pentaho ETL -&gt; PostgreSQL DWH -&gt; Power BI)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Scope: data already loaded to DWH facts &amp; dimensions by client. Blue = input hours, black = formula.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="9" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Work package</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Requirement section(s)</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Scope in Power BI architecture</t>
+        </is>
+      </c>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Best case (h)</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr">
+        <is>
+          <t>Estimated (h)</t>
+        </is>
+      </c>
+      <c r="G4" s="9" t="inlineStr">
+        <is>
+          <t>Worst case (h)</t>
+        </is>
+      </c>
+      <c r="H4" s="9" t="inlineStr">
+        <is>
+          <t>% of base</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="10" t="inlineStr">
+        <is>
+          <t>Discovery &amp; clarification</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D5" s="10" t="inlineStr">
+        <is>
+          <t>Report definitions, review of DWH schema (facts/dims), definitions of service %, via, KT weight</t>
+        </is>
+      </c>
+      <c r="E5" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="F5" s="29" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" s="29" t="n">
+        <v>18</v>
+      </c>
+      <c r="H5" s="30">
+        <f>F5/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="10" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Semantic model</t>
+        </is>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
+        <is>
+          <t>0, 9</t>
+        </is>
+      </c>
+      <c r="D6" s="10" t="inlineStr">
+        <is>
+          <t>PostgreSQL connection, relationships, date dimension, security, model performance</t>
+        </is>
+      </c>
+      <c r="E6" s="29" t="n">
+        <v>18</v>
+      </c>
+      <c r="F6" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="G6" s="29" t="n">
+        <v>32</v>
+      </c>
+      <c r="H6" s="30">
+        <f>F6/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="10" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="10" t="inlineStr">
+        <is>
+          <t>Configurable target engine</t>
+        </is>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>1, 9</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="inlineStr">
+        <is>
+          <t>Target table in DWH, what-if / field parameters for target days (4/5/6/7+), DAX measures</t>
+        </is>
+      </c>
+      <c r="E7" s="29" t="n">
+        <v>16</v>
+      </c>
+      <c r="F7" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="G7" s="29" t="n">
+        <v>28</v>
+      </c>
+      <c r="H7" s="30">
+        <f>F7/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Service % &amp; target achievement reports</t>
+        </is>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>1, 2</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="inlineStr">
+        <is>
+          <t>Source/destination/route/via/business service %, target %, actual %, variation %, ranking</t>
+        </is>
+      </c>
+      <c r="E8" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="F8" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="G8" s="29" t="n">
+        <v>40</v>
+      </c>
+      <c r="H8" s="30">
+        <f>F8/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="10" t="inlineStr">
+        <is>
+          <t>Delay &amp; journey analysis, drill-through</t>
+        </is>
+      </c>
+      <c r="C9" s="10" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D9" s="10" t="inlineStr">
+        <is>
+          <t>Stage-wise delay, route -&gt; stage -&gt; LR -&gt; reason drill-through, remarks</t>
+        </is>
+      </c>
+      <c r="E9" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="F9" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="G9" s="29" t="n">
+        <v>40</v>
+      </c>
+      <c r="H9" s="30">
+        <f>F9/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>LR search &amp; consignor/consignee analytics</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="D10" s="10" t="inlineStr">
+        <is>
+          <t>LR journey page, consignor/consignee reports and variation vs target</t>
+        </is>
+      </c>
+      <c r="E10" s="29" t="n">
+        <v>16</v>
+      </c>
+      <c r="F10" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="G10" s="29" t="n">
+        <v>28</v>
+      </c>
+      <c r="H10" s="30">
+        <f>F10/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="10" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Period-wise &amp; comparison reports</t>
+        </is>
+      </c>
+      <c r="C11" s="10" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="D11" s="10" t="inlineStr">
+        <is>
+          <t>Weekly/10-day/15-day/monthly/yearly, custom period, current vs previous (DAX time intelligence)</t>
+        </is>
+      </c>
+      <c r="E11" s="29" t="n">
+        <v>10</v>
+      </c>
+      <c r="F11" s="29" t="n">
+        <v>14</v>
+      </c>
+      <c r="G11" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="H11" s="30">
+        <f>F11/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Booking -&gt; main hub dispatch</t>
+        </is>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="D12" s="10" t="inlineStr">
+        <is>
+          <t>Receipt/dispatch times, pending/delayed/dispatched LR ageing, source &amp; hub performance</t>
+        </is>
+      </c>
+      <c r="E12" s="29" t="n">
+        <v>18</v>
+      </c>
+      <c r="F12" s="29" t="n">
+        <v>22</v>
+      </c>
+      <c r="G12" s="29" t="n">
+        <v>30</v>
+      </c>
+      <c r="H12" s="30">
+        <f>F12/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="10" t="inlineStr">
+        <is>
+          <t>Live reports</t>
+        </is>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="inlineStr">
+        <is>
+          <t>DirectQuery or near-real-time refresh on DWH (Pentaho pulls SRD API); 6 live reports</t>
+        </is>
+      </c>
+      <c r="E13" s="29" t="n">
+        <v>18</v>
+      </c>
+      <c r="F13" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="G13" s="29" t="n">
+        <v>40</v>
+      </c>
+      <c r="H13" s="30">
+        <f>F13/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="10" t="inlineStr">
+        <is>
+          <t>Improvement suggestions</t>
+        </is>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="inlineStr">
+        <is>
+          <t>SQL/Python job writing route/stage/LR suggestions to DWH; surfaced in Power BI</t>
+        </is>
+      </c>
+      <c r="E14" s="29" t="n">
+        <v>12</v>
+      </c>
+      <c r="F14" s="29" t="n">
+        <v>16</v>
+      </c>
+      <c r="G14" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="H14" s="30">
+        <f>F14/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="10" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="10" t="inlineStr">
+        <is>
+          <t>ML delay-risk scoring (optional)</t>
+        </is>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>Existing</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="inlineStr">
+        <is>
+          <t>Python scoring job writes risk &amp; top factors to DWH; Power BI reads. Drop if not required</t>
+        </is>
+      </c>
+      <c r="E15" s="29" t="n">
+        <v>14</v>
+      </c>
+      <c r="F15" s="29" t="n">
+        <v>20</v>
+      </c>
+      <c r="G15" s="29" t="n">
+        <v>28</v>
+      </c>
+      <c r="H15" s="30">
+        <f>F15/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="10" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="10" t="inlineStr">
+        <is>
+          <t>Slicers, filters &amp; export</t>
+        </is>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="inlineStr">
+        <is>
+          <t>Slicers for period/source/destination/via/business/consignor/consignee/LR, export</t>
+        </is>
+      </c>
+      <c r="E16" s="29" t="n">
+        <v>6</v>
+      </c>
+      <c r="F16" s="29" t="n">
+        <v>8</v>
+      </c>
+      <c r="G16" s="29" t="n">
+        <v>12</v>
+      </c>
+      <c r="H16" s="30">
+        <f>F16/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="10" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Testing, UAT, gateway, refresh, publish</t>
+        </is>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="inlineStr">
+        <is>
+          <t>UAT cycle, on-prem gateway, scheduled refresh, Power BI Service deployment, documentation</t>
+        </is>
+      </c>
+      <c r="E17" s="29" t="n">
+        <v>18</v>
+      </c>
+      <c r="F17" s="29" t="n">
+        <v>24</v>
+      </c>
+      <c r="G17" s="29" t="n">
+        <v>32</v>
+      </c>
+      <c r="H17" s="30">
+        <f>F17/$F$18</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="n"/>
+      <c r="B18" s="13" t="inlineStr">
+        <is>
+          <t>Base total (before buffer)</t>
+        </is>
+      </c>
+      <c r="C18" s="13" t="n"/>
+      <c r="D18" s="13" t="n"/>
+      <c r="E18" s="31">
+        <f>SUM(E5:E17)</f>
+        <v/>
+      </c>
+      <c r="F18" s="31">
+        <f>SUM(F5:F17)</f>
+        <v/>
+      </c>
+      <c r="G18" s="31">
+        <f>SUM(G5:G17)</f>
+        <v/>
+      </c>
+      <c r="H18" s="32">
+        <f>SUM(H5:H17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="13" t="n"/>
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>Contingency buffer</t>
+        </is>
+      </c>
+      <c r="C19" s="13" t="n"/>
+      <c r="D19" s="13" t="inlineStr">
+        <is>
+          <t>Linked to Assumptions!B3 (same 100 h buffer)</t>
+        </is>
+      </c>
+      <c r="E19" s="33">
+        <f>Assumptions!$B$3</f>
+        <v/>
+      </c>
+      <c r="F19" s="33">
+        <f>Assumptions!$B$3</f>
+        <v/>
+      </c>
+      <c r="G19" s="33">
+        <f>Assumptions!$B$3</f>
+        <v/>
+      </c>
+      <c r="H19" s="13" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="n"/>
+      <c r="B20" s="17" t="inlineStr">
+        <is>
+          <t>GRAND TOTAL (with buffer)</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="34">
+        <f>E18+E19</f>
+        <v/>
+      </c>
+      <c r="F20" s="34">
+        <f>F18+F19</f>
+        <v/>
+      </c>
+      <c r="G20" s="34">
+        <f>G18+G19</f>
+        <v/>
+      </c>
+      <c r="H20" s="17" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="23" t="inlineStr">
+        <is>
+          <t>Assumptions</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="B23" s="24" t="inlineStr">
+        <is>
+          <t>1. Data engineering (Pentaho ETL, staging, PostgreSQL DWH facts/dimensions) is done by the client and excluded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="B24" s="24" t="inlineStr">
+        <is>
+          <t>2. DWH already contains LR, consignor, consignee, via, hub, business and journey-stage timestamps; otherwise ETL effort returns.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t>3. Power BI cannot run the scikit-learn/SHAP model directly; ML is a Python scoring job writing to the DWH (row 11, optional).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="B26" s="24" t="inlineStr">
+        <is>
+          <t>4. Live API data is pulled by Pentaho into the DWH every few minutes; Power BI uses DirectQuery. Streaming datasets would change effort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="28" customHeight="1">
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>5. Excluded: Power BI Pro/Premium licensing, hosting, user management beyond basic row-level security.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="28" customHeight="1">
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>6. Best/worst case columns are judgement-based ranges around the estimate, not statistical bounds.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B26:H26"/>
+    <mergeCell ref="B27:H27"/>
+    <mergeCell ref="B24:H24"/>
+    <mergeCell ref="B25:H25"/>
+    <mergeCell ref="B28:H28"/>
+    <mergeCell ref="B23:H23"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -810,16 +1629,16 @@
           <t>Requirement clarification, SRD data &amp; API mapping, definitions (service %, via, KT weight)</t>
         </is>
       </c>
-      <c r="E5" s="11" t="n">
+      <c r="E5" s="29" t="n">
         <v>16</v>
       </c>
-      <c r="F5" s="11" t="n">
+      <c r="F5" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="G5" s="11" t="n">
+      <c r="G5" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="H5" s="12">
+      <c r="H5" s="30">
         <f>F5/$F$18</f>
         <v/>
       </c>
@@ -843,16 +1662,16 @@
           <t>Ingestion/ETL, LR-level schema (LR, consignor, consignee, via, hub, business, stage timestamps), cleaning &amp; validation</t>
         </is>
       </c>
-      <c r="E6" s="11" t="n">
+      <c r="E6" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="F6" s="11" t="n">
+      <c r="F6" s="29" t="n">
         <v>40</v>
       </c>
-      <c r="G6" s="11" t="n">
+      <c r="G6" s="29" t="n">
         <v>55</v>
       </c>
-      <c r="H6" s="12">
+      <c r="H6" s="30">
         <f>F6/$F$18</f>
         <v/>
       </c>
@@ -876,16 +1695,16 @@
           <t>Per route / source-destination benchmark TAT, target-days (4/5/6/7+), config UI, no hard-coded rules</t>
         </is>
       </c>
-      <c r="E7" s="11" t="n">
+      <c r="E7" s="29" t="n">
         <v>22</v>
       </c>
-      <c r="F7" s="11" t="n">
+      <c r="F7" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="G7" s="11" t="n">
+      <c r="G7" s="29" t="n">
         <v>36</v>
       </c>
-      <c r="H7" s="12">
+      <c r="H7" s="30">
         <f>F7/$F$18</f>
         <v/>
       </c>
@@ -909,16 +1728,16 @@
           <t>Source/destination/route/via/business service %, target %, actual %, variation %, ranked delays</t>
         </is>
       </c>
-      <c r="E8" s="11" t="n">
+      <c r="E8" s="29" t="n">
         <v>26</v>
       </c>
-      <c r="F8" s="11" t="n">
+      <c r="F8" s="29" t="n">
         <v>32</v>
       </c>
-      <c r="G8" s="11" t="n">
+      <c r="G8" s="29" t="n">
         <v>42</v>
       </c>
-      <c r="H8" s="12">
+      <c r="H8" s="30">
         <f>F8/$F$18</f>
         <v/>
       </c>
@@ -942,16 +1761,16 @@
           <t>Stage-level delay logic (booking→delivery), route→stage→LR→reason drill-down, delay remarks</t>
         </is>
       </c>
-      <c r="E9" s="11" t="n">
+      <c r="E9" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="F9" s="11" t="n">
+      <c r="F9" s="29" t="n">
         <v>36</v>
       </c>
-      <c r="G9" s="11" t="n">
+      <c r="G9" s="29" t="n">
         <v>46</v>
       </c>
-      <c r="H9" s="12">
+      <c r="H9" s="30">
         <f>F9/$F$18</f>
         <v/>
       </c>
@@ -975,16 +1794,16 @@
           <t>LR journey timeline, consignor/consignee search &amp; service % vs target, source/dest/route/period drill-down</t>
         </is>
       </c>
-      <c r="E10" s="11" t="n">
+      <c r="E10" s="29" t="n">
         <v>22</v>
       </c>
-      <c r="F10" s="11" t="n">
+      <c r="F10" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="G10" s="11" t="n">
+      <c r="G10" s="29" t="n">
         <v>36</v>
       </c>
-      <c r="H10" s="12">
+      <c r="H10" s="30">
         <f>F10/$F$18</f>
         <v/>
       </c>
@@ -1008,16 +1827,16 @@
           <t>Weekly/10-day/15-day/monthly/yearly views, custom period, current vs previous comparison</t>
         </is>
       </c>
-      <c r="E11" s="11" t="n">
+      <c r="E11" s="29" t="n">
         <v>16</v>
       </c>
-      <c r="F11" s="11" t="n">
+      <c r="F11" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="G11" s="11" t="n">
+      <c r="G11" s="29" t="n">
         <v>26</v>
       </c>
-      <c r="H11" s="12">
+      <c r="H11" s="30">
         <f>F11/$F$18</f>
         <v/>
       </c>
@@ -1041,16 +1860,16 @@
           <t>Receipt/dispatch time calc, pending/delayed/dispatched LR ageing, source &amp; hub performance</t>
         </is>
       </c>
-      <c r="E12" s="11" t="n">
+      <c r="E12" s="29" t="n">
         <v>22</v>
       </c>
-      <c r="F12" s="11" t="n">
+      <c r="F12" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="G12" s="11" t="n">
+      <c r="G12" s="29" t="n">
         <v>36</v>
       </c>
-      <c r="H12" s="12">
+      <c r="H12" s="30">
         <f>F12/$F$18</f>
         <v/>
       </c>
@@ -1074,16 +1893,16 @@
           <t>API client/auth, polling &amp; caching, 6 live reports (bookings, lag/lead, target, KT weight, godown stock, hub movement)</t>
         </is>
       </c>
-      <c r="E13" s="11" t="n">
+      <c r="E13" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="F13" s="11" t="n">
+      <c r="F13" s="29" t="n">
         <v>36</v>
       </c>
-      <c r="G13" s="11" t="n">
+      <c r="G13" s="29" t="n">
         <v>56</v>
       </c>
-      <c r="H13" s="12">
+      <c r="H13" s="30">
         <f>F13/$F$18</f>
         <v/>
       </c>
@@ -1107,16 +1926,16 @@
           <t>Move rule engine from network level to route/stage/LR-level suggestions</t>
         </is>
       </c>
-      <c r="E14" s="11" t="n">
+      <c r="E14" s="29" t="n">
         <v>16</v>
       </c>
-      <c r="F14" s="11" t="n">
+      <c r="F14" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="G14" s="11" t="n">
+      <c r="G14" s="29" t="n">
         <v>26</v>
       </c>
-      <c r="H14" s="12">
+      <c r="H14" s="30">
         <f>F14/$F$18</f>
         <v/>
       </c>
@@ -1140,16 +1959,16 @@
           <t>Retrain on real data, update features, SHAP &amp; what-if adjustments</t>
         </is>
       </c>
-      <c r="E15" s="11" t="n">
+      <c r="E15" s="29" t="n">
         <v>14</v>
       </c>
-      <c r="F15" s="11" t="n">
+      <c r="F15" s="29" t="n">
         <v>20</v>
       </c>
-      <c r="G15" s="11" t="n">
+      <c r="G15" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="H15" s="12">
+      <c r="H15" s="30">
         <f>F15/$F$18</f>
         <v/>
       </c>
@@ -1173,16 +1992,16 @@
           <t>Filters for via/business/consignor/consignee/LR, CSV/Excel export, standard report table</t>
         </is>
       </c>
-      <c r="E16" s="11" t="n">
+      <c r="E16" s="29" t="n">
         <v>10</v>
       </c>
-      <c r="F16" s="11" t="n">
+      <c r="F16" s="29" t="n">
         <v>12</v>
       </c>
-      <c r="G16" s="11" t="n">
+      <c r="G16" s="29" t="n">
         <v>16</v>
       </c>
-      <c r="H16" s="12">
+      <c r="H16" s="30">
         <f>F16/$F$18</f>
         <v/>
       </c>
@@ -1206,16 +2025,16 @@
           <t>Unit tests, UAT cycle, deployment, user documentation</t>
         </is>
       </c>
-      <c r="E17" s="11" t="n">
+      <c r="E17" s="29" t="n">
         <v>24</v>
       </c>
-      <c r="F17" s="11" t="n">
+      <c r="F17" s="29" t="n">
         <v>30</v>
       </c>
-      <c r="G17" s="11" t="n">
+      <c r="G17" s="29" t="n">
         <v>40</v>
       </c>
-      <c r="H17" s="12">
+      <c r="H17" s="30">
         <f>F17/$F$18</f>
         <v/>
       </c>
@@ -1229,19 +2048,19 @@
       </c>
       <c r="C18" s="13" t="n"/>
       <c r="D18" s="13" t="n"/>
-      <c r="E18" s="14">
+      <c r="E18" s="31">
         <f>SUM(E5:E17)</f>
         <v/>
       </c>
-      <c r="F18" s="14">
+      <c r="F18" s="31">
         <f>SUM(F5:F17)</f>
         <v/>
       </c>
-      <c r="G18" s="14">
+      <c r="G18" s="31">
         <f>SUM(G5:G17)</f>
         <v/>
       </c>
-      <c r="H18" s="15">
+      <c r="H18" s="32">
         <f>SUM(H5:H17)</f>
         <v/>
       </c>
@@ -1259,15 +2078,15 @@
           <t>Additional buffer agreed with stakeholder; covers unknown data quality, API spec, UAT rework, scope creep</t>
         </is>
       </c>
-      <c r="E19" s="16">
+      <c r="E19" s="33">
         <f>Assumptions!$B$3</f>
         <v/>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="33">
         <f>Assumptions!$B$3</f>
         <v/>
       </c>
-      <c r="G19" s="16">
+      <c r="G19" s="33">
         <f>Assumptions!$B$3</f>
         <v/>
       </c>
@@ -1282,15 +2101,15 @@
       </c>
       <c r="C20" s="17" t="n"/>
       <c r="D20" s="17" t="n"/>
-      <c r="E20" s="18">
+      <c r="E20" s="34">
         <f>E18+E19</f>
         <v/>
       </c>
-      <c r="F20" s="18">
+      <c r="F20" s="34">
         <f>F18+F19</f>
         <v/>
       </c>
-      <c r="G20" s="18">
+      <c r="G20" s="34">
         <f>G18+G19</f>
         <v/>
       </c>
@@ -1301,7 +2120,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1484,7 +2303,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>